<commit_message>
modificado proyecto final y creado power bi
</commit_message>
<xml_diff>
--- a/datos_limpios/libros_limpios.xlsx
+++ b/datos_limpios/libros_limpios.xlsx
@@ -491,7 +491,7 @@
       </c>
       <c r="C3" t="inlineStr">
         <is>
-          <t>Buenaventura de Bonet</t>
+          <t>Buenaventura De Bonet</t>
         </is>
       </c>
       <c r="D3" t="n">
@@ -521,7 +521,7 @@
       </c>
       <c r="C4" t="inlineStr">
         <is>
-          <t>Ileana AntÃ³n-AndrÃ©s</t>
+          <t>Ileana Antón-Andrés</t>
         </is>
       </c>
       <c r="D4" t="n">
@@ -551,7 +551,7 @@
       </c>
       <c r="C5" t="inlineStr">
         <is>
-          <t>CÃ©sar Guerrero Vazquez</t>
+          <t>César Guerrero Vazquez</t>
         </is>
       </c>
       <c r="D5" t="n">
@@ -611,7 +611,7 @@
       </c>
       <c r="C7" t="inlineStr">
         <is>
-          <t>Jacobo del Agudo</t>
+          <t>Jacobo Del Agudo</t>
         </is>
       </c>
       <c r="D7" t="n">
@@ -731,7 +731,7 @@
       </c>
       <c r="C11" t="inlineStr">
         <is>
-          <t>Soraya NÃºÃ±ez Lamas</t>
+          <t>Soraya Núñez Lamas</t>
         </is>
       </c>
       <c r="D11" t="n">
@@ -761,7 +761,7 @@
       </c>
       <c r="C12" t="inlineStr">
         <is>
-          <t>PÃ¡nfilo Segovia Casanovas</t>
+          <t>Pánfilo Segovia Casanovas</t>
         </is>
       </c>
       <c r="D12" t="n">
@@ -821,7 +821,7 @@
       </c>
       <c r="C14" t="inlineStr">
         <is>
-          <t>Celia BaÃ±os-Arroyo</t>
+          <t>Celia Baños-Arroyo</t>
         </is>
       </c>
       <c r="D14" t="n">
@@ -851,7 +851,7 @@
       </c>
       <c r="C15" t="inlineStr">
         <is>
-          <t>Rolando del Bernal</t>
+          <t>Rolando Del Bernal</t>
         </is>
       </c>
       <c r="D15" t="n">
@@ -881,7 +881,7 @@
       </c>
       <c r="C16" t="inlineStr">
         <is>
-          <t>Toribio de Pinto</t>
+          <t>Toribio De Pinto</t>
         </is>
       </c>
       <c r="D16" t="n">
@@ -911,7 +911,7 @@
       </c>
       <c r="C17" t="inlineStr">
         <is>
-          <t>Javi PatiÃ±o-CÃ¡novas</t>
+          <t>Javi Patiño-Cánovas</t>
         </is>
       </c>
       <c r="D17" t="n">
@@ -1001,7 +1001,7 @@
       </c>
       <c r="C20" t="inlineStr">
         <is>
-          <t>JerÃ³nimo Pino Lerma</t>
+          <t>Jerónimo Pino Lerma</t>
         </is>
       </c>
       <c r="D20" t="n">
@@ -1031,7 +1031,7 @@
       </c>
       <c r="C21" t="inlineStr">
         <is>
-          <t>Constanza del Barba</t>
+          <t>Constanza Del Barba</t>
         </is>
       </c>
       <c r="D21" t="n">
@@ -1061,7 +1061,7 @@
       </c>
       <c r="C22" t="inlineStr">
         <is>
-          <t>Segismundo de Moles</t>
+          <t>Segismundo De Moles</t>
         </is>
       </c>
       <c r="D22" t="n">
@@ -1091,7 +1091,7 @@
       </c>
       <c r="C23" t="inlineStr">
         <is>
-          <t>Edelmira Batalla GalvÃ¡n</t>
+          <t>Edelmira Batalla Galván</t>
         </is>
       </c>
       <c r="D23" t="n">
@@ -1181,7 +1181,7 @@
       </c>
       <c r="C26" t="inlineStr">
         <is>
-          <t>Buenaventura Huerta-JÃ³dar</t>
+          <t>Buenaventura Huerta-Jódar</t>
         </is>
       </c>
       <c r="D26" t="n">
@@ -1211,7 +1211,7 @@
       </c>
       <c r="C27" t="inlineStr">
         <is>
-          <t>InÃ©s Pujol-Paredes</t>
+          <t>Inés Pujol-Paredes</t>
         </is>
       </c>
       <c r="D27" t="n">
@@ -1241,7 +1241,7 @@
       </c>
       <c r="C28" t="inlineStr">
         <is>
-          <t>Bruno del Bou</t>
+          <t>Bruno Del Bou</t>
         </is>
       </c>
       <c r="D28" t="n">
@@ -1301,7 +1301,7 @@
       </c>
       <c r="C30" t="inlineStr">
         <is>
-          <t>Ruy Roca BartolomÃ©</t>
+          <t>Ruy Roca Bartolomé</t>
         </is>
       </c>
       <c r="D30" t="n">
@@ -1331,7 +1331,7 @@
       </c>
       <c r="C31" t="inlineStr">
         <is>
-          <t>Francisca SolÃ© Ãngel</t>
+          <t>Francisca Solé Ángel</t>
         </is>
       </c>
       <c r="D31" t="n">
@@ -1361,7 +1361,7 @@
       </c>
       <c r="C32" t="inlineStr">
         <is>
-          <t>Leonel Alberdi-CarbÃ³</t>
+          <t>Leonel Alberdi-Carbó</t>
         </is>
       </c>
       <c r="D32" t="n">
@@ -1391,7 +1391,7 @@
       </c>
       <c r="C33" t="inlineStr">
         <is>
-          <t>Pili del Nieto</t>
+          <t>Pili Del Nieto</t>
         </is>
       </c>
       <c r="D33" t="n">
@@ -1481,7 +1481,7 @@
       </c>
       <c r="C36" t="inlineStr">
         <is>
-          <t>JosÃ© Luis Camino MartÃ­n</t>
+          <t>José Luis Camino Martín</t>
         </is>
       </c>
       <c r="D36" t="n">
@@ -1511,7 +1511,7 @@
       </c>
       <c r="C37" t="inlineStr">
         <is>
-          <t>MarÃ­a Fernanda Flor</t>
+          <t>María Fernanda Flor</t>
         </is>
       </c>
       <c r="D37" t="n">
@@ -1541,7 +1541,7 @@
       </c>
       <c r="C38" t="inlineStr">
         <is>
-          <t>Glauco CuÃ©llar Abascal</t>
+          <t>Glauco Cuéllar Abascal</t>
         </is>
       </c>
       <c r="D38" t="n">
@@ -1571,7 +1571,7 @@
       </c>
       <c r="C39" t="inlineStr">
         <is>
-          <t>Etelvina Laura Aliaga CaparrÃ³s</t>
+          <t>Etelvina Laura Aliaga Caparrós</t>
         </is>
       </c>
       <c r="D39" t="n">
@@ -1601,7 +1601,7 @@
       </c>
       <c r="C40" t="inlineStr">
         <is>
-          <t>Valeria MelÃ©ndez Heras</t>
+          <t>Valeria Meléndez Heras</t>
         </is>
       </c>
       <c r="D40" t="n">
@@ -1631,7 +1631,7 @@
       </c>
       <c r="C41" t="inlineStr">
         <is>
-          <t>Dionisio BermÃºdez Boada</t>
+          <t>Dionisio Bermúdez Boada</t>
         </is>
       </c>
       <c r="D41" t="n">
@@ -1661,7 +1661,7 @@
       </c>
       <c r="C42" t="inlineStr">
         <is>
-          <t>Sabina BayÃ³n Casas</t>
+          <t>Sabina Bayón Casas</t>
         </is>
       </c>
       <c r="D42" t="n">
@@ -1721,7 +1721,7 @@
       </c>
       <c r="C44" t="inlineStr">
         <is>
-          <t>Juan Luis Rocha-GalÃ¡n</t>
+          <t>Juan Luis Rocha-Galán</t>
         </is>
       </c>
       <c r="D44" t="n">
@@ -1751,7 +1751,7 @@
       </c>
       <c r="C45" t="inlineStr">
         <is>
-          <t>Priscila de Mesa</t>
+          <t>Priscila De Mesa</t>
         </is>
       </c>
       <c r="D45" t="n">
@@ -1781,7 +1781,7 @@
       </c>
       <c r="C46" t="inlineStr">
         <is>
-          <t>Nazaret Perea RÃ­os</t>
+          <t>Nazaret Perea Ríos</t>
         </is>
       </c>
       <c r="D46" t="n">
@@ -1841,7 +1841,7 @@
       </c>
       <c r="C48" t="inlineStr">
         <is>
-          <t>Daniel de Neira</t>
+          <t>Daniel De Neira</t>
         </is>
       </c>
       <c r="D48" t="n">
@@ -1871,7 +1871,7 @@
       </c>
       <c r="C49" t="inlineStr">
         <is>
-          <t>Macario Grau GimÃ©nez</t>
+          <t>Macario Grau Giménez</t>
         </is>
       </c>
       <c r="D49" t="n">
@@ -1901,7 +1901,7 @@
       </c>
       <c r="C50" t="inlineStr">
         <is>
-          <t>AndrÃ©s Felipe Barral Granados</t>
+          <t>Andrés Felipe Barral Granados</t>
         </is>
       </c>
       <c r="D50" t="n">
@@ -1931,7 +1931,7 @@
       </c>
       <c r="C51" t="inlineStr">
         <is>
-          <t>VÃ­ctor Angulo Murillo</t>
+          <t>Víctor Angulo Murillo</t>
         </is>
       </c>
       <c r="D51" t="n">
@@ -1961,7 +1961,7 @@
       </c>
       <c r="C52" t="inlineStr">
         <is>
-          <t>JosÃ© Ãngel GÃ¡rate Lopez</t>
+          <t>José Ángel Gárate Lopez</t>
         </is>
       </c>
       <c r="D52" t="n">
@@ -1991,7 +1991,7 @@
       </c>
       <c r="C53" t="inlineStr">
         <is>
-          <t>Clotilde CatalÃ¡n SuÃ¡rez</t>
+          <t>Clotilde Catalán Suárez</t>
         </is>
       </c>
       <c r="D53" t="n">
@@ -2021,7 +2021,7 @@
       </c>
       <c r="C54" t="inlineStr">
         <is>
-          <t>Ruben del RamÃ­rez</t>
+          <t>Ruben Del Ramírez</t>
         </is>
       </c>
       <c r="D54" t="n">
@@ -2171,7 +2171,7 @@
       </c>
       <c r="C59" t="inlineStr">
         <is>
-          <t>Clemente de Sanabria</t>
+          <t>Clemente De Sanabria</t>
         </is>
       </c>
       <c r="D59" t="n">
@@ -2201,7 +2201,7 @@
       </c>
       <c r="C60" t="inlineStr">
         <is>
-          <t>HÃ©ctor EspaÃ±ol Lopez</t>
+          <t>Héctor Español Lopez</t>
         </is>
       </c>
       <c r="D60" t="n">
@@ -2261,7 +2261,7 @@
       </c>
       <c r="C62" t="inlineStr">
         <is>
-          <t>Ariel de Alcolea</t>
+          <t>Ariel De Alcolea</t>
         </is>
       </c>
       <c r="D62" t="n">
@@ -2291,7 +2291,7 @@
       </c>
       <c r="C63" t="inlineStr">
         <is>
-          <t>Renato GuzmÃ¡n Delgado</t>
+          <t>Renato Guzmán Delgado</t>
         </is>
       </c>
       <c r="D63" t="n">
@@ -2321,7 +2321,7 @@
       </c>
       <c r="C64" t="inlineStr">
         <is>
-          <t>Julieta Teruel GarcÃ­a</t>
+          <t>Julieta Teruel García</t>
         </is>
       </c>
       <c r="D64" t="n">
@@ -2351,7 +2351,7 @@
       </c>
       <c r="C65" t="inlineStr">
         <is>
-          <t>Yaiza Barral CÃ³zar</t>
+          <t>Yaiza Barral Cózar</t>
         </is>
       </c>
       <c r="D65" t="n">
@@ -2411,7 +2411,7 @@
       </c>
       <c r="C67" t="inlineStr">
         <is>
-          <t>EloÃ­sa Rocha Torrecilla</t>
+          <t>Eloísa Rocha Torrecilla</t>
         </is>
       </c>
       <c r="D67" t="n">
@@ -2531,7 +2531,7 @@
       </c>
       <c r="C71" t="inlineStr">
         <is>
-          <t>Camila BarberÃ¡</t>
+          <t>Camila Barberá</t>
         </is>
       </c>
       <c r="D71" t="n">
@@ -2621,7 +2621,7 @@
       </c>
       <c r="C74" t="inlineStr">
         <is>
-          <t>Azeneth Hoz AriÃ±o</t>
+          <t>Azeneth Hoz Ariño</t>
         </is>
       </c>
       <c r="D74" t="n">
@@ -2651,7 +2651,7 @@
       </c>
       <c r="C75" t="inlineStr">
         <is>
-          <t>Anita Hortensia YÃ¡Ã±ez Molina</t>
+          <t>Anita Hortensia Yáñez Molina</t>
         </is>
       </c>
       <c r="D75" t="n">
@@ -2681,7 +2681,7 @@
       </c>
       <c r="C76" t="inlineStr">
         <is>
-          <t>Cristian Miralles-GÃ³mez</t>
+          <t>Cristian Miralles-Gómez</t>
         </is>
       </c>
       <c r="D76" t="n">
@@ -2711,7 +2711,7 @@
       </c>
       <c r="C77" t="inlineStr">
         <is>
-          <t>Hector Castro-MarÃ­n</t>
+          <t>Hector Castro-Marín</t>
         </is>
       </c>
       <c r="D77" t="n">
@@ -2741,7 +2741,7 @@
       </c>
       <c r="C78" t="inlineStr">
         <is>
-          <t>Estela Belmonte AgustÃ­</t>
+          <t>Estela Belmonte Agustí</t>
         </is>
       </c>
       <c r="D78" t="n">
@@ -2771,7 +2771,7 @@
       </c>
       <c r="C79" t="inlineStr">
         <is>
-          <t>MarÃ­a Ãngeles Cabo BeltrÃ¡n</t>
+          <t>María Ángeles Cabo Beltrán</t>
         </is>
       </c>
       <c r="D79" t="n">
@@ -2801,7 +2801,7 @@
       </c>
       <c r="C80" t="inlineStr">
         <is>
-          <t>Clotilde del Cazorla</t>
+          <t>Clotilde Del Cazorla</t>
         </is>
       </c>
       <c r="D80" t="n">
@@ -2861,7 +2861,7 @@
       </c>
       <c r="C82" t="inlineStr">
         <is>
-          <t>Elodia Cruz RÃ­os</t>
+          <t>Elodia Cruz Ríos</t>
         </is>
       </c>
       <c r="D82" t="n">
@@ -2891,7 +2891,7 @@
       </c>
       <c r="C83" t="inlineStr">
         <is>
-          <t>Ofelia del Ãngel</t>
+          <t>Ofelia Del Ángel</t>
         </is>
       </c>
       <c r="D83" t="n">
@@ -2921,7 +2921,7 @@
       </c>
       <c r="C84" t="inlineStr">
         <is>
-          <t>Nazario MarÃ­ Calleja</t>
+          <t>Nazario Marí Calleja</t>
         </is>
       </c>
       <c r="D84" t="n">
@@ -2981,7 +2981,7 @@
       </c>
       <c r="C86" t="inlineStr">
         <is>
-          <t>Calixta del LujÃ¡n</t>
+          <t>Calixta Del Luján</t>
         </is>
       </c>
       <c r="D86" t="n">
@@ -3041,7 +3041,7 @@
       </c>
       <c r="C88" t="inlineStr">
         <is>
-          <t>JosÃ© Antonio Torres-Iglesias</t>
+          <t>José Antonio Torres-Iglesias</t>
         </is>
       </c>
       <c r="D88" t="n">
@@ -3101,7 +3101,7 @@
       </c>
       <c r="C90" t="inlineStr">
         <is>
-          <t>Abel MÃºgica Castrillo</t>
+          <t>Abel Múgica Castrillo</t>
         </is>
       </c>
       <c r="D90" t="n">
@@ -3161,7 +3161,7 @@
       </c>
       <c r="C92" t="inlineStr">
         <is>
-          <t>Adelia de Benet</t>
+          <t>Adelia De Benet</t>
         </is>
       </c>
       <c r="D92" t="n">
@@ -3191,7 +3191,7 @@
       </c>
       <c r="C93" t="inlineStr">
         <is>
-          <t>Leandro Araujo PeirÃ³</t>
+          <t>Leandro Araujo Peiró</t>
         </is>
       </c>
       <c r="D93" t="n">
@@ -3281,7 +3281,7 @@
       </c>
       <c r="C96" t="inlineStr">
         <is>
-          <t>Vinicio PallarÃ¨s Gallo</t>
+          <t>Vinicio Pallarès Gallo</t>
         </is>
       </c>
       <c r="D96" t="n">
@@ -3311,7 +3311,7 @@
       </c>
       <c r="C97" t="inlineStr">
         <is>
-          <t>Nazario de Otero</t>
+          <t>Nazario De Otero</t>
         </is>
       </c>
       <c r="D97" t="n">
@@ -3341,7 +3341,7 @@
       </c>
       <c r="C98" t="inlineStr">
         <is>
-          <t>VerÃ³nica del Cortes</t>
+          <t>Verónica Del Cortes</t>
         </is>
       </c>
       <c r="D98" t="n">
@@ -3371,7 +3371,7 @@
       </c>
       <c r="C99" t="inlineStr">
         <is>
-          <t>Toni de Elorza</t>
+          <t>Toni De Elorza</t>
         </is>
       </c>
       <c r="D99" t="n">
@@ -3401,7 +3401,7 @@
       </c>
       <c r="C100" t="inlineStr">
         <is>
-          <t>Aitana Escobar MÃ¡rquez</t>
+          <t>Aitana Escobar Márquez</t>
         </is>
       </c>
       <c r="D100" t="n">
@@ -3461,7 +3461,7 @@
       </c>
       <c r="C102" t="inlineStr">
         <is>
-          <t>Rufino Campoy PiÃ±eiro</t>
+          <t>Rufino Campoy Piñeiro</t>
         </is>
       </c>
       <c r="D102" t="n">
@@ -3491,7 +3491,7 @@
       </c>
       <c r="C103" t="inlineStr">
         <is>
-          <t>Timoteo Sosa GirÃ³n</t>
+          <t>Timoteo Sosa Girón</t>
         </is>
       </c>
       <c r="D103" t="n">
@@ -3521,7 +3521,7 @@
       </c>
       <c r="C104" t="inlineStr">
         <is>
-          <t>Sebastian SeguÃ­</t>
+          <t>Sebastian Seguí</t>
         </is>
       </c>
       <c r="D104" t="n">
@@ -3551,7 +3551,7 @@
       </c>
       <c r="C105" t="inlineStr">
         <is>
-          <t>EncarnaciÃ³n GoÃ±i Gisbert</t>
+          <t>Encarnación Goñi Gisbert</t>
         </is>
       </c>
       <c r="D105" t="n">
@@ -3611,7 +3611,7 @@
       </c>
       <c r="C107" t="inlineStr">
         <is>
-          <t>Eligia BaÃ±os Lorenzo</t>
+          <t>Eligia Baños Lorenzo</t>
         </is>
       </c>
       <c r="D107" t="n">
@@ -3671,7 +3671,7 @@
       </c>
       <c r="C109" t="inlineStr">
         <is>
-          <t>Eusebia de Carlos</t>
+          <t>Eusebia De Carlos</t>
         </is>
       </c>
       <c r="D109" t="n">
@@ -3791,7 +3791,7 @@
       </c>
       <c r="C113" t="inlineStr">
         <is>
-          <t>Ximena FalcÃ³n IÃ±iguez</t>
+          <t>Ximena Falcón Iñiguez</t>
         </is>
       </c>
       <c r="D113" t="n">
@@ -3821,7 +3821,7 @@
       </c>
       <c r="C114" t="inlineStr">
         <is>
-          <t>Paulino Rubio AbellÃ¡n</t>
+          <t>Paulino Rubio Abellán</t>
         </is>
       </c>
       <c r="D114" t="n">
@@ -3851,7 +3851,7 @@
       </c>
       <c r="C115" t="inlineStr">
         <is>
-          <t>Ãngela Figueras</t>
+          <t>Ángela Figueras</t>
         </is>
       </c>
       <c r="D115" t="n">
@@ -3911,7 +3911,7 @@
       </c>
       <c r="C117" t="inlineStr">
         <is>
-          <t>EstefanÃ­a Narcisa Casanovas Mas</t>
+          <t>Estefanía Narcisa Casanovas Mas</t>
         </is>
       </c>
       <c r="D117" t="n">
@@ -3971,7 +3971,7 @@
       </c>
       <c r="C119" t="inlineStr">
         <is>
-          <t>Graciana MarquÃ©s CastejÃ³n</t>
+          <t>Graciana Marqués Castejón</t>
         </is>
       </c>
       <c r="D119" t="n">
@@ -4031,7 +4031,7 @@
       </c>
       <c r="C121" t="inlineStr">
         <is>
-          <t>Mario MascarÃ³ Ramis</t>
+          <t>Mario Mascaró Ramis</t>
         </is>
       </c>
       <c r="D121" t="n">
@@ -4061,7 +4061,7 @@
       </c>
       <c r="C122" t="inlineStr">
         <is>
-          <t>Serafina de Mateu</t>
+          <t>Serafina De Mateu</t>
         </is>
       </c>
       <c r="D122" t="n">
@@ -4121,7 +4121,7 @@
       </c>
       <c r="C124" t="inlineStr">
         <is>
-          <t>Isaura GarcÃ­a Vicente</t>
+          <t>Isaura García Vicente</t>
         </is>
       </c>
       <c r="D124" t="n">
@@ -4151,7 +4151,7 @@
       </c>
       <c r="C125" t="inlineStr">
         <is>
-          <t>Rosalina DomÃ©nech Blazquez</t>
+          <t>Rosalina Doménech Blazquez</t>
         </is>
       </c>
       <c r="D125" t="n">
@@ -4181,7 +4181,7 @@
       </c>
       <c r="C126" t="inlineStr">
         <is>
-          <t>JosÃ© Ãngel Natanael Naranjo Bueno</t>
+          <t>José Ángel Natanael Naranjo Bueno</t>
         </is>
       </c>
       <c r="D126" t="n">
@@ -4211,7 +4211,7 @@
       </c>
       <c r="C127" t="inlineStr">
         <is>
-          <t>Nicodemo del Gomila</t>
+          <t>Nicodemo Del Gomila</t>
         </is>
       </c>
       <c r="D127" t="n">
@@ -4331,7 +4331,7 @@
       </c>
       <c r="C131" t="inlineStr">
         <is>
-          <t>Gloria HervÃ¡s Coloma</t>
+          <t>Gloria Hervás Coloma</t>
         </is>
       </c>
       <c r="D131" t="n">
@@ -4361,7 +4361,7 @@
       </c>
       <c r="C132" t="inlineStr">
         <is>
-          <t>Victoriano Campillo RodrÃ­guez</t>
+          <t>Victoriano Campillo Rodríguez</t>
         </is>
       </c>
       <c r="D132" t="n">
@@ -4391,7 +4391,7 @@
       </c>
       <c r="C133" t="inlineStr">
         <is>
-          <t>Chus del AyllÃ³n</t>
+          <t>Chus Del Ayllón</t>
         </is>
       </c>
       <c r="D133" t="n">
@@ -4421,7 +4421,7 @@
       </c>
       <c r="C134" t="inlineStr">
         <is>
-          <t>Diana de Sastre</t>
+          <t>Diana De Sastre</t>
         </is>
       </c>
       <c r="D134" t="n">
@@ -4481,7 +4481,7 @@
       </c>
       <c r="C136" t="inlineStr">
         <is>
-          <t>MarÃ­a JosÃ© Vargas Roldan</t>
+          <t>María José Vargas Roldan</t>
         </is>
       </c>
       <c r="D136" t="n">
@@ -4511,7 +4511,7 @@
       </c>
       <c r="C137" t="inlineStr">
         <is>
-          <t>Itziar de Taboada</t>
+          <t>Itziar De Taboada</t>
         </is>
       </c>
       <c r="D137" t="n">
@@ -4631,7 +4631,7 @@
       </c>
       <c r="C141" t="inlineStr">
         <is>
-          <t>ElÃ­as del Montenegro</t>
+          <t>Elías Del Montenegro</t>
         </is>
       </c>
       <c r="D141" t="n">
@@ -4661,7 +4661,7 @@
       </c>
       <c r="C142" t="inlineStr">
         <is>
-          <t>Anita de Contreras</t>
+          <t>Anita De Contreras</t>
         </is>
       </c>
       <c r="D142" t="n">
@@ -4691,7 +4691,7 @@
       </c>
       <c r="C143" t="inlineStr">
         <is>
-          <t>Gregorio de Gargallo</t>
+          <t>Gregorio De Gargallo</t>
         </is>
       </c>
       <c r="D143" t="n">
@@ -4721,7 +4721,7 @@
       </c>
       <c r="C144" t="inlineStr">
         <is>
-          <t>HipÃ³lito RamÃ³n Muro</t>
+          <t>Hipólito Ramón Muro</t>
         </is>
       </c>
       <c r="D144" t="n">
@@ -4751,7 +4751,7 @@
       </c>
       <c r="C145" t="inlineStr">
         <is>
-          <t>Josefa del Barrios</t>
+          <t>Josefa Del Barrios</t>
         </is>
       </c>
       <c r="D145" t="n">
@@ -4841,7 +4841,7 @@
       </c>
       <c r="C148" t="inlineStr">
         <is>
-          <t>Adelaida Ortiz MartÃ­n</t>
+          <t>Adelaida Ortiz Martín</t>
         </is>
       </c>
       <c r="D148" t="n">
@@ -4871,7 +4871,7 @@
       </c>
       <c r="C149" t="inlineStr">
         <is>
-          <t>Tamara Rius GimÃ©nez</t>
+          <t>Tamara Rius Giménez</t>
         </is>
       </c>
       <c r="D149" t="n">
@@ -4991,7 +4991,7 @@
       </c>
       <c r="C153" t="inlineStr">
         <is>
-          <t>MarÃ­a Amores Prada</t>
+          <t>María Amores Prada</t>
         </is>
       </c>
       <c r="D153" t="n">
@@ -5081,7 +5081,7 @@
       </c>
       <c r="C156" t="inlineStr">
         <is>
-          <t>Eladio Pinilla MorÃ¡n</t>
+          <t>Eladio Pinilla Morán</t>
         </is>
       </c>
       <c r="D156" t="n">
@@ -5141,7 +5141,7 @@
       </c>
       <c r="C158" t="inlineStr">
         <is>
-          <t>PÃ­a Pinilla Lobo</t>
+          <t>Pía Pinilla Lobo</t>
         </is>
       </c>
       <c r="D158" t="n">
@@ -5231,7 +5231,7 @@
       </c>
       <c r="C161" t="inlineStr">
         <is>
-          <t>Moreno de Arjona</t>
+          <t>Moreno De Arjona</t>
         </is>
       </c>
       <c r="D161" t="n">
@@ -5291,7 +5291,7 @@
       </c>
       <c r="C163" t="inlineStr">
         <is>
-          <t>Calista Dafne Cases SÃ¡enz</t>
+          <t>Calista Dafne Cases Sáenz</t>
         </is>
       </c>
       <c r="D163" t="n">
@@ -5381,7 +5381,7 @@
       </c>
       <c r="C166" t="inlineStr">
         <is>
-          <t>MarÃ­a Dolores Piedad CarbÃ³ CÃ©spedes</t>
+          <t>María Dolores Piedad Carbó Céspedes</t>
         </is>
       </c>
       <c r="D166" t="n">
@@ -5411,7 +5411,7 @@
       </c>
       <c r="C167" t="inlineStr">
         <is>
-          <t>Baltasar Luis Miguel AmigÃ³ Mesa</t>
+          <t>Baltasar Luis Miguel Amigó Mesa</t>
         </is>
       </c>
       <c r="D167" t="n">
@@ -5561,7 +5561,7 @@
       </c>
       <c r="C172" t="inlineStr">
         <is>
-          <t>InÃ©s del BayÃ³n</t>
+          <t>Inés Del Bayón</t>
         </is>
       </c>
       <c r="D172" t="n">
@@ -5681,7 +5681,7 @@
       </c>
       <c r="C176" t="inlineStr">
         <is>
-          <t>Isaac EcheverrÃ­a VÃ©lez</t>
+          <t>Isaac Echeverría Vélez</t>
         </is>
       </c>
       <c r="D176" t="n">
@@ -5711,7 +5711,7 @@
       </c>
       <c r="C177" t="inlineStr">
         <is>
-          <t>Mario TomÃ¡s-Sola</t>
+          <t>Mario Tomás-Sola</t>
         </is>
       </c>
       <c r="D177" t="n">
@@ -5771,7 +5771,7 @@
       </c>
       <c r="C179" t="inlineStr">
         <is>
-          <t>Severo de Lorenzo</t>
+          <t>Severo De Lorenzo</t>
         </is>
       </c>
       <c r="D179" t="n">
@@ -5921,7 +5921,7 @@
       </c>
       <c r="C184" t="inlineStr">
         <is>
-          <t>Adelina de Boada</t>
+          <t>Adelina De Boada</t>
         </is>
       </c>
       <c r="D184" t="n">
@@ -5951,7 +5951,7 @@
       </c>
       <c r="C185" t="inlineStr">
         <is>
-          <t>PlÃ¡cido del Torres</t>
+          <t>Plácido Del Torres</t>
         </is>
       </c>
       <c r="D185" t="n">
@@ -5981,7 +5981,7 @@
       </c>
       <c r="C186" t="inlineStr">
         <is>
-          <t>PurificaciÃ³n de Tamayo</t>
+          <t>Purificación De Tamayo</t>
         </is>
       </c>
       <c r="D186" t="n">
@@ -6011,7 +6011,7 @@
       </c>
       <c r="C187" t="inlineStr">
         <is>
-          <t>Jacinta Alemany BuendÃ­a</t>
+          <t>Jacinta Alemany Buendía</t>
         </is>
       </c>
       <c r="D187" t="n">
@@ -6071,7 +6071,7 @@
       </c>
       <c r="C189" t="inlineStr">
         <is>
-          <t>Flor SÃ¡enz-NÃºÃ±ez</t>
+          <t>Flor Sáenz-Núñez</t>
         </is>
       </c>
       <c r="D189" t="n">
@@ -6161,7 +6161,7 @@
       </c>
       <c r="C192" t="inlineStr">
         <is>
-          <t>Benito de Moles</t>
+          <t>Benito De Moles</t>
         </is>
       </c>
       <c r="D192" t="n">
@@ -6221,7 +6221,7 @@
       </c>
       <c r="C194" t="inlineStr">
         <is>
-          <t>Rafael TomÃ©</t>
+          <t>Rafael Tomé</t>
         </is>
       </c>
       <c r="D194" t="n">
@@ -6311,7 +6311,7 @@
       </c>
       <c r="C197" t="inlineStr">
         <is>
-          <t>Geraldo de Mate</t>
+          <t>Geraldo De Mate</t>
         </is>
       </c>
       <c r="D197" t="n">
@@ -6341,7 +6341,7 @@
       </c>
       <c r="C198" t="inlineStr">
         <is>
-          <t>Paulino CastaÃ±eda LledÃ³</t>
+          <t>Paulino Castañeda Lledó</t>
         </is>
       </c>
       <c r="D198" t="n">
@@ -6401,7 +6401,7 @@
       </c>
       <c r="C200" t="inlineStr">
         <is>
-          <t>Aroa Alberola LuÃ­s</t>
+          <t>Aroa Alberola Luís</t>
         </is>
       </c>
       <c r="D200" t="n">
@@ -6431,7 +6431,7 @@
       </c>
       <c r="C201" t="inlineStr">
         <is>
-          <t>Julia Saez NiÃ±o</t>
+          <t>Julia Saez Niño</t>
         </is>
       </c>
       <c r="D201" t="n">

</xml_diff>